<commit_message>
Optimizadores establecidos junto con filtros en rectangulares
</commit_message>
<xml_diff>
--- a/Krec5x4.xlsx
+++ b/Krec5x4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\topopt3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743E5BDA-0258-437E-A380-1BF2826072EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E239AC77-355B-4117-B04E-58889524DCEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82F11E43-85F1-4E4E-AF48-846E60F2CAD0}"/>
+    <workbookView xWindow="3696" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{82F11E43-85F1-4E4E-AF48-846E60F2CAD0}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -403,12 +403,110 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2439A4C4-214E-4114-A65D-16E5348289A8}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A2:BH61"/>
+  <dimension ref="A1:BH61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="60" width="5.77734375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:60" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>1</v>
+      </c>
+      <c r="D1">
+        <v>1</v>
+      </c>
+      <c r="E1">
+        <v>0</v>
+      </c>
+      <c r="F1">
+        <v>0</v>
+      </c>
+      <c r="G1">
+        <v>0</v>
+      </c>
+      <c r="H1">
+        <v>0</v>
+      </c>
+      <c r="I1">
+        <v>1</v>
+      </c>
+      <c r="J1">
+        <v>1</v>
+      </c>
+      <c r="K1">
+        <v>1</v>
+      </c>
+      <c r="L1">
+        <v>1</v>
+      </c>
+      <c r="M1">
+        <v>0</v>
+      </c>
+      <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
+        <v>0</v>
+      </c>
+      <c r="P1">
+        <v>0</v>
+      </c>
+      <c r="Q1">
+        <v>0</v>
+      </c>
+      <c r="R1">
+        <v>0</v>
+      </c>
+      <c r="S1">
+        <v>0</v>
+      </c>
+      <c r="T1">
+        <v>0</v>
+      </c>
+      <c r="U1">
+        <v>0</v>
+      </c>
+      <c r="V1">
+        <v>0</v>
+      </c>
+      <c r="W1">
+        <v>0</v>
+      </c>
+      <c r="X1">
+        <v>0</v>
+      </c>
+      <c r="Y1">
+        <v>0</v>
+      </c>
+      <c r="Z1">
+        <v>0</v>
+      </c>
+      <c r="AA1">
+        <v>0</v>
+      </c>
+      <c r="AB1">
+        <v>0</v>
+      </c>
+      <c r="AC1">
+        <v>0</v>
+      </c>
+      <c r="AD1">
+        <v>0</v>
+      </c>
+      <c r="AE1">
+        <v>0</v>
+      </c>
+      <c r="AF1">
+        <v>0</v>
+      </c>
+    </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
@@ -435,10 +533,10 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -447,10 +545,10 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -599,16 +697,16 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -617,16 +715,16 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -799,28 +897,28 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -957,28 +1055,28 @@
     </row>
     <row r="5" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1169,28 +1267,28 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6">
         <v>0</v>
@@ -1327,16 +1425,16 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -1363,16 +1461,16 @@
         <v>1</v>
       </c>
       <c r="O7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7">
         <v>0</v>
@@ -1521,16 +1619,16 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -1539,10 +1637,10 @@
         <v>0</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8">
         <v>1</v>
@@ -1551,16 +1649,16 @@
         <v>1</v>
       </c>
       <c r="Q8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U8">
         <v>0</v>
@@ -1685,40 +1783,40 @@
     </row>
     <row r="9" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M9">
         <v>0</v>
@@ -1727,16 +1825,16 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9">
         <v>1</v>
@@ -1867,16 +1965,16 @@
     </row>
     <row r="10" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1885,22 +1983,22 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M10">
         <v>0</v>
@@ -2049,46 +2147,46 @@
     </row>
     <row r="11" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O11">
         <v>0</v>
@@ -2103,16 +2201,16 @@
         <v>1</v>
       </c>
       <c r="S11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W11">
         <v>0</v>
@@ -2237,16 +2335,16 @@
         <v>1</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -2255,16 +2353,16 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12">
         <v>2</v>
@@ -2279,16 +2377,16 @@
         <v>0</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U12">
         <v>1</v>
@@ -2297,10 +2395,10 @@
         <v>1</v>
       </c>
       <c r="W12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y12">
         <v>0</v>
@@ -2413,10 +2511,10 @@
     </row>
     <row r="13" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -2425,16 +2523,16 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -2449,16 +2547,16 @@
         <v>2</v>
       </c>
       <c r="M13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -2467,16 +2565,16 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13">
         <v>1</v>
@@ -2595,28 +2693,28 @@
     </row>
     <row r="14" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -2649,28 +2747,28 @@
         <v>0</v>
       </c>
       <c r="S14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA14">
         <v>0</v>
@@ -2777,16 +2875,16 @@
     </row>
     <row r="15" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2795,10 +2893,10 @@
         <v>1</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -2807,16 +2905,16 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O15">
         <v>2</v>
@@ -2843,16 +2941,16 @@
         <v>1</v>
       </c>
       <c r="W15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA15">
         <v>0</v>
@@ -2965,16 +3063,16 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -3001,16 +3099,16 @@
         <v>2</v>
       </c>
       <c r="O16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S16">
         <v>0</v>
@@ -3019,10 +3117,10 @@
         <v>0</v>
       </c>
       <c r="U16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W16">
         <v>1</v>
@@ -3031,16 +3129,16 @@
         <v>1</v>
       </c>
       <c r="Y16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC16">
         <v>0</v>
@@ -3147,46 +3245,46 @@
         <v>0</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P17">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q17">
         <v>2</v>
@@ -3195,10 +3293,10 @@
         <v>2</v>
       </c>
       <c r="S17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U17">
         <v>0</v>
@@ -3207,16 +3305,16 @@
         <v>0</v>
       </c>
       <c r="W17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA17">
         <v>1</v>
@@ -3335,16 +3433,16 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>1</v>
@@ -3353,10 +3451,10 @@
         <v>1</v>
       </c>
       <c r="K18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18">
         <v>0</v>
@@ -3365,16 +3463,16 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S18">
         <v>2</v>
@@ -3401,16 +3499,16 @@
         <v>1</v>
       </c>
       <c r="AA18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE18">
         <v>0</v>
@@ -3517,16 +3615,16 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I19">
         <v>1</v>
@@ -3535,40 +3633,40 @@
         <v>1</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q19">
+        <v>2</v>
+      </c>
+      <c r="R19">
+        <v>2</v>
+      </c>
+      <c r="S19">
         <v>4</v>
       </c>
-      <c r="R19">
+      <c r="T19">
         <v>4</v>
       </c>
-      <c r="S19">
-        <v>2</v>
-      </c>
-      <c r="T19">
-        <v>2</v>
-      </c>
       <c r="U19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -3705,10 +3803,10 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20">
         <v>1</v>
@@ -3717,16 +3815,16 @@
         <v>1</v>
       </c>
       <c r="K20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20">
         <v>0</v>
@@ -3741,16 +3839,16 @@
         <v>2</v>
       </c>
       <c r="S20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W20">
         <v>0</v>
@@ -3759,16 +3857,16 @@
         <v>0</v>
       </c>
       <c r="Y20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC20">
         <v>1</v>
@@ -3887,40 +3985,40 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S21">
         <v>2</v>
@@ -3929,16 +4027,16 @@
         <v>2</v>
       </c>
       <c r="U21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y21">
         <v>0</v>
@@ -3953,16 +4051,16 @@
         <v>1</v>
       </c>
       <c r="AC21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG21">
         <v>0</v>
@@ -4087,16 +4185,16 @@
         <v>1</v>
       </c>
       <c r="M22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q22">
         <v>0</v>
@@ -4105,16 +4203,16 @@
         <v>0</v>
       </c>
       <c r="S22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W22">
         <v>2</v>
@@ -4129,16 +4227,16 @@
         <v>0</v>
       </c>
       <c r="AA22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE22">
         <v>1</v>
@@ -4263,10 +4361,10 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23">
         <v>1</v>
@@ -4275,10 +4373,10 @@
         <v>1</v>
       </c>
       <c r="O23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q23">
         <v>0</v>
@@ -4317,10 +4415,10 @@
         <v>0</v>
       </c>
       <c r="AC23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE23">
         <v>1</v>
@@ -4445,16 +4543,16 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24">
         <v>1</v>
@@ -4481,16 +4579,16 @@
         <v>2</v>
       </c>
       <c r="W24">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X24">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA24">
         <v>0</v>
@@ -4499,10 +4597,10 @@
         <v>0</v>
       </c>
       <c r="AC24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE24">
         <v>1</v>
@@ -4627,58 +4725,58 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W25">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X25">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC25">
         <v>0</v>
@@ -4687,10 +4785,10 @@
         <v>0</v>
       </c>
       <c r="AE25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG25">
         <v>2</v>
@@ -4815,16 +4913,16 @@
         <v>0</v>
       </c>
       <c r="M26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q26">
         <v>1</v>
@@ -4833,10 +4931,10 @@
         <v>1</v>
       </c>
       <c r="S26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U26">
         <v>0</v>
@@ -4845,22 +4943,22 @@
         <v>0</v>
       </c>
       <c r="W26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Z26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AA26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC26">
         <v>0</v>
@@ -4997,16 +5095,16 @@
         <v>0</v>
       </c>
       <c r="M27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q27">
         <v>1</v>
@@ -5015,28 +5113,28 @@
         <v>1</v>
       </c>
       <c r="S27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Z27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AA27">
         <v>2</v>
@@ -5045,10 +5143,10 @@
         <v>2</v>
       </c>
       <c r="AC27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE27">
         <v>0</v>
@@ -5185,28 +5283,28 @@
         <v>0</v>
       </c>
       <c r="O28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -5215,22 +5313,22 @@
         <v>0</v>
       </c>
       <c r="Y28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE28">
         <v>0</v>
@@ -5367,16 +5465,16 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S29">
         <v>1</v>
@@ -5385,28 +5483,28 @@
         <v>1</v>
       </c>
       <c r="U29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA29">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AB29">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC29">
         <v>2</v>
@@ -5415,10 +5513,10 @@
         <v>2</v>
       </c>
       <c r="AE29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG29">
         <v>0</v>
@@ -5555,10 +5653,10 @@
         <v>0</v>
       </c>
       <c r="Q30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S30">
         <v>1</v>
@@ -5567,16 +5665,16 @@
         <v>1</v>
       </c>
       <c r="U30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y30">
         <v>0</v>
@@ -5585,10 +5683,10 @@
         <v>0</v>
       </c>
       <c r="AA30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC30">
         <v>2</v>
@@ -5597,10 +5695,10 @@
         <v>2</v>
       </c>
       <c r="AE30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG30">
         <v>0</v>
@@ -5737,28 +5835,28 @@
         <v>0</v>
       </c>
       <c r="Q31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y31">
         <v>0</v>
@@ -5767,22 +5865,22 @@
         <v>0</v>
       </c>
       <c r="AA31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG31">
         <v>0</v>
@@ -5955,16 +6053,16 @@
         <v>0</v>
       </c>
       <c r="AC32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG32">
         <v>2</v>

</xml_diff>